<commit_message>
updated with some revisions
</commit_message>
<xml_diff>
--- a/AxialSeamount_2023_metadata_BCO-DMO.xlsx
+++ b/AxialSeamount_2023_metadata_BCO-DMO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/skhu/Desktop/Projects/axial-amplicons-2023/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{548F0C63-5832-E54B-842D-F7BE266C91BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AFE2DC6-2BEC-C443-80AF-C9E40C2A7214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1320" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{3697DE8D-83FB-6B46-9496-DA5921FA009A}"/>
+    <workbookView xWindow="39000" yWindow="500" windowWidth="47020" windowHeight="17640" xr2:uid="{3697DE8D-83FB-6B46-9496-DA5921FA009A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet3" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1685" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1690" uniqueCount="335">
   <si>
     <t>Accession</t>
   </si>
@@ -1040,12 +1040,15 @@
   <si>
     <t>longitude</t>
   </si>
+  <si>
+    <t>DATE</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1085,6 +1088,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1106,7 +1122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1124,6 +1140,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1458,13 +1478,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28977624-7CB7-E04C-BC3D-9861C4B1C988}">
-  <dimension ref="A1:V91"/>
+  <dimension ref="A1:W91"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:23" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1531,8 +1551,11 @@
       <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W1" s="9" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -1599,8 +1622,11 @@
       <c r="V2" s="6">
         <v>-129.97996670000001</v>
       </c>
-    </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W2" s="10">
+        <v>44752</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>37</v>
       </c>
@@ -1667,8 +1693,11 @@
       <c r="V3" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W3" s="11">
+        <v>44751</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>45</v>
       </c>
@@ -1735,8 +1764,11 @@
       <c r="V4" s="6">
         <v>-129.97996670000001</v>
       </c>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W4" s="10">
+        <v>44752</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>48</v>
       </c>
@@ -1803,8 +1835,11 @@
       <c r="V5" s="6">
         <v>-129.97996670000001</v>
       </c>
-    </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W5" s="10">
+        <v>44752</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>51</v>
       </c>
@@ -1871,8 +1906,11 @@
       <c r="V6" s="7">
         <v>-130.04949999999999</v>
       </c>
-    </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W6" s="10">
+        <v>45128</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>55</v>
       </c>
@@ -1939,8 +1977,11 @@
       <c r="V7" s="7">
         <v>-130.04949999999999</v>
       </c>
-    </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W7" s="10">
+        <v>45128</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>57</v>
       </c>
@@ -2007,8 +2048,11 @@
       <c r="V8" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W8" s="11">
+        <v>44751</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>61</v>
       </c>
@@ -2075,8 +2119,11 @@
       <c r="V9" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W9" s="11">
+        <v>44751</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>64</v>
       </c>
@@ -2140,8 +2187,11 @@
       <c r="U10" s="5" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W10" s="12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>75</v>
       </c>
@@ -2205,8 +2255,11 @@
       <c r="U11" s="5" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W11" s="12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>78</v>
       </c>
@@ -2265,8 +2318,11 @@
       <c r="U12" s="5" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W12" s="12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>82</v>
       </c>
@@ -2333,8 +2389,11 @@
       <c r="V13" s="7">
         <v>-129.989225</v>
       </c>
-    </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W13" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>89</v>
       </c>
@@ -2401,8 +2460,11 @@
       <c r="V14" s="7">
         <v>-129.97906499999999</v>
       </c>
-    </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W14" s="10">
+        <v>45129</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>94</v>
       </c>
@@ -2469,8 +2531,11 @@
       <c r="V15" s="7">
         <v>-129.98233200000001</v>
       </c>
-    </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W15" s="10">
+        <v>45128</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>101</v>
       </c>
@@ -2537,8 +2602,11 @@
       <c r="V16" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W16" s="10">
+        <v>45125</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>106</v>
       </c>
@@ -2605,8 +2673,11 @@
       <c r="V17" s="7">
         <v>-129.989225</v>
       </c>
-    </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W17" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>109</v>
       </c>
@@ -2673,8 +2744,11 @@
       <c r="V18" s="7">
         <v>-129.989225</v>
       </c>
-    </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W18" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>113</v>
       </c>
@@ -2741,8 +2815,11 @@
       <c r="V19" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W19" s="10">
+        <v>45127</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>118</v>
       </c>
@@ -2809,8 +2886,11 @@
       <c r="V20" s="7">
         <v>-129.98233200000001</v>
       </c>
-    </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W20" s="10">
+        <v>45128</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>120</v>
       </c>
@@ -2877,8 +2957,11 @@
       <c r="V21" s="7">
         <v>-129.99296100000001</v>
       </c>
-    </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W21" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>124</v>
       </c>
@@ -2945,8 +3028,11 @@
       <c r="V22" s="7">
         <v>-129.99296100000001</v>
       </c>
-    </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W22" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>126</v>
       </c>
@@ -3013,8 +3099,11 @@
       <c r="V23" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W23" s="10">
+        <v>45125</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>128</v>
       </c>
@@ -3081,8 +3170,11 @@
       <c r="V24" s="7">
         <v>-129.97906499999999</v>
       </c>
-    </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W24" s="10">
+        <v>45129</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>130</v>
       </c>
@@ -3149,8 +3241,11 @@
       <c r="V25" s="7">
         <v>-130.01327739999999</v>
       </c>
-    </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W25" s="10">
+        <v>45132</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>135</v>
       </c>
@@ -3217,8 +3312,11 @@
       <c r="V26" s="7">
         <v>-130.01327739999999</v>
       </c>
-    </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W26" s="10">
+        <v>45132</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>137</v>
       </c>
@@ -3285,8 +3383,11 @@
       <c r="V27" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W27" s="10">
+        <v>45127</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>139</v>
       </c>
@@ -3353,8 +3454,11 @@
       <c r="V28" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W28" s="10">
+        <v>45127</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>142</v>
       </c>
@@ -3421,8 +3525,11 @@
       <c r="V29" s="7">
         <v>-130.01348899999999</v>
       </c>
-    </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W29" s="10">
+        <v>45126</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>147</v>
       </c>
@@ -3489,8 +3596,11 @@
       <c r="V30" s="6">
         <v>-129.97996670000001</v>
       </c>
-    </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W30" s="10">
+        <v>45129</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>151</v>
       </c>
@@ -3557,8 +3667,11 @@
       <c r="V31" s="7">
         <v>-129.989225</v>
       </c>
-    </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W31" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>154</v>
       </c>
@@ -3625,8 +3738,11 @@
       <c r="V32" s="7">
         <v>-129.989225</v>
       </c>
-    </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W32" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>156</v>
       </c>
@@ -3693,8 +3809,11 @@
       <c r="V33" s="7">
         <v>-129.97906499999999</v>
       </c>
-    </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W33" s="10">
+        <v>45129</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>159</v>
       </c>
@@ -3761,8 +3880,11 @@
       <c r="V34" s="7">
         <v>-129.97906499999999</v>
       </c>
-    </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W34" s="10">
+        <v>45129</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>161</v>
       </c>
@@ -3829,8 +3951,11 @@
       <c r="V35" s="7">
         <v>-130.01327739999999</v>
       </c>
-    </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W35" s="10">
+        <v>45132</v>
+      </c>
+    </row>
+    <row r="36" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>164</v>
       </c>
@@ -3897,8 +4022,11 @@
       <c r="V36" s="7">
         <v>-130.01327739999999</v>
       </c>
-    </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W36" s="10">
+        <v>45132</v>
+      </c>
+    </row>
+    <row r="37" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>166</v>
       </c>
@@ -3965,8 +4093,11 @@
       <c r="V37" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W37" s="10">
+        <v>45127</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>169</v>
       </c>
@@ -4033,8 +4164,11 @@
       <c r="V38" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W38" s="10">
+        <v>45127</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>171</v>
       </c>
@@ -4101,8 +4235,11 @@
       <c r="V39" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W39" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>174</v>
       </c>
@@ -4169,8 +4306,11 @@
       <c r="V40" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W40" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>176</v>
       </c>
@@ -4237,8 +4377,11 @@
       <c r="V41" s="7">
         <v>-129.98233200000001</v>
       </c>
-    </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W41" s="10">
+        <v>45130</v>
+      </c>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>180</v>
       </c>
@@ -4305,8 +4448,11 @@
       <c r="V42" s="7">
         <v>-129.98233200000001</v>
       </c>
-    </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W42" s="10">
+        <v>45130</v>
+      </c>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>182</v>
       </c>
@@ -4373,8 +4519,11 @@
       <c r="V43" s="7">
         <v>-130.01348899999999</v>
       </c>
-    </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W43" s="10">
+        <v>45126</v>
+      </c>
+    </row>
+    <row r="44" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>185</v>
       </c>
@@ -4441,8 +4590,11 @@
       <c r="V44" s="7">
         <v>-130.01328520000001</v>
       </c>
-    </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W44" s="10">
+        <v>45132</v>
+      </c>
+    </row>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>192</v>
       </c>
@@ -4509,8 +4661,11 @@
       <c r="V45" s="7">
         <v>-130.01348899999999</v>
       </c>
-    </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W45" s="10">
+        <v>45126</v>
+      </c>
+    </row>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>194</v>
       </c>
@@ -4577,8 +4732,11 @@
       <c r="V46" s="7">
         <v>-130.01382409999999</v>
       </c>
-    </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W46" s="10">
+        <v>45132</v>
+      </c>
+    </row>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>197</v>
       </c>
@@ -4645,8 +4803,11 @@
       <c r="V47" s="7">
         <v>-129.98195699999999</v>
       </c>
-    </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W47" s="10">
+        <v>45130</v>
+      </c>
+    </row>
+    <row r="48" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>201</v>
       </c>
@@ -4713,8 +4874,11 @@
       <c r="V48" s="6">
         <v>-129.97996670000001</v>
       </c>
-    </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W48" s="10">
+        <v>45129</v>
+      </c>
+    </row>
+    <row r="49" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>203</v>
       </c>
@@ -4781,8 +4945,11 @@
       <c r="V49" s="7">
         <v>-129.97906499999999</v>
       </c>
-    </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W49" s="10">
+        <v>45129</v>
+      </c>
+    </row>
+    <row r="50" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>206</v>
       </c>
@@ -4849,8 +5016,11 @@
       <c r="V50" s="7">
         <v>-129.97906499999999</v>
       </c>
-    </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W50" s="10">
+        <v>45129</v>
+      </c>
+    </row>
+    <row r="51" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>208</v>
       </c>
@@ -4914,8 +5084,11 @@
       <c r="U51" s="5" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W51" s="12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="52" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>211</v>
       </c>
@@ -4982,8 +5155,11 @@
       <c r="V52" s="7">
         <v>-129.98233200000001</v>
       </c>
-    </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W52" s="10">
+        <v>45128</v>
+      </c>
+    </row>
+    <row r="53" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>214</v>
       </c>
@@ -5050,8 +5226,11 @@
       <c r="V53" s="7">
         <v>-130.01348899999999</v>
       </c>
-    </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W53" s="10">
+        <v>45126</v>
+      </c>
+    </row>
+    <row r="54" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>216</v>
       </c>
@@ -5118,8 +5297,11 @@
       <c r="V54" s="6">
         <v>-129.97996670000001</v>
       </c>
-    </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W54" s="10">
+        <v>45129</v>
+      </c>
+    </row>
+    <row r="55" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>218</v>
       </c>
@@ -5186,8 +5368,11 @@
       <c r="V55" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W55" s="10">
+        <v>45126</v>
+      </c>
+    </row>
+    <row r="56" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>222</v>
       </c>
@@ -5254,8 +5439,11 @@
       <c r="V56" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W56" s="10">
+        <v>45126</v>
+      </c>
+    </row>
+    <row r="57" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>225</v>
       </c>
@@ -5322,8 +5510,11 @@
       <c r="V57" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W57" s="10">
+        <v>45126</v>
+      </c>
+    </row>
+    <row r="58" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>228</v>
       </c>
@@ -5390,8 +5581,11 @@
       <c r="V58" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W58" s="10">
+        <v>45126</v>
+      </c>
+    </row>
+    <row r="59" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>231</v>
       </c>
@@ -5458,8 +5652,11 @@
       <c r="V59" s="7">
         <v>-129.989225</v>
       </c>
-    </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W59" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="60" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>234</v>
       </c>
@@ -5526,8 +5723,11 @@
       <c r="V60" s="7">
         <v>-129.989225</v>
       </c>
-    </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W60" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="61" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>237</v>
       </c>
@@ -5594,8 +5794,11 @@
       <c r="V61" s="6">
         <v>-129.97996670000001</v>
       </c>
-    </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W61" s="10">
+        <v>45129</v>
+      </c>
+    </row>
+    <row r="62" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>239</v>
       </c>
@@ -5662,8 +5865,11 @@
       <c r="V62" s="7">
         <v>-130.01327739999999</v>
       </c>
-    </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W62" s="10">
+        <v>45132</v>
+      </c>
+    </row>
+    <row r="63" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>242</v>
       </c>
@@ -5730,8 +5936,11 @@
       <c r="V63" s="7">
         <v>-130.01327739999999</v>
       </c>
-    </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W63" s="10">
+        <v>45132</v>
+      </c>
+    </row>
+    <row r="64" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>245</v>
       </c>
@@ -5798,8 +6007,11 @@
       <c r="V64" s="7">
         <v>-129.97906499999999</v>
       </c>
-    </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W64" s="10">
+        <v>45129</v>
+      </c>
+    </row>
+    <row r="65" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>248</v>
       </c>
@@ -5866,8 +6078,11 @@
       <c r="V65" s="7">
         <v>-129.97906499999999</v>
       </c>
-    </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W65" s="10">
+        <v>45129</v>
+      </c>
+    </row>
+    <row r="66" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>250</v>
       </c>
@@ -5934,8 +6149,11 @@
       <c r="V66" s="7">
         <v>-129.98195699999999</v>
       </c>
-    </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W66" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="67" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>254</v>
       </c>
@@ -6002,8 +6220,11 @@
       <c r="V67" s="7">
         <v>-129.98233200000001</v>
       </c>
-    </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W67" s="10">
+        <v>45130</v>
+      </c>
+    </row>
+    <row r="68" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>256</v>
       </c>
@@ -6070,8 +6291,11 @@
       <c r="V68" s="7">
         <v>-129.98233200000001</v>
       </c>
-    </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W68" s="10">
+        <v>45130</v>
+      </c>
+    </row>
+    <row r="69" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>258</v>
       </c>
@@ -6138,8 +6362,11 @@
       <c r="V69" s="7">
         <v>-129.98233200000001</v>
       </c>
-    </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W69" s="10">
+        <v>45130</v>
+      </c>
+    </row>
+    <row r="70" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>261</v>
       </c>
@@ -6206,8 +6433,11 @@
       <c r="V70" s="7">
         <v>-129.98233200000001</v>
       </c>
-    </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W70" s="10">
+        <v>45130</v>
+      </c>
+    </row>
+    <row r="71" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>264</v>
       </c>
@@ -6274,8 +6504,11 @@
       <c r="V71" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W71" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="72" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>267</v>
       </c>
@@ -6342,8 +6575,11 @@
       <c r="V72" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W72" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="73" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>270</v>
       </c>
@@ -6410,8 +6646,11 @@
       <c r="V73" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W73" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="74" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>273</v>
       </c>
@@ -6478,8 +6717,11 @@
       <c r="V74" s="7">
         <v>-130.01406800000001</v>
       </c>
-    </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W74" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="75" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>275</v>
       </c>
@@ -6546,8 +6788,11 @@
       <c r="V75" s="7">
         <v>-129.99296100000001</v>
       </c>
-    </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W75" s="10">
+        <v>45131</v>
+      </c>
+    </row>
+    <row r="76" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>278</v>
       </c>
@@ -6614,8 +6859,11 @@
       <c r="V76" s="7">
         <v>-129.98233200000001</v>
       </c>
-    </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W76" s="10">
+        <v>45128</v>
+      </c>
+    </row>
+    <row r="77" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>280</v>
       </c>
@@ -6682,8 +6930,11 @@
       <c r="V77" s="7">
         <v>-129.98233200000001</v>
       </c>
-    </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W77" s="10">
+        <v>45128</v>
+      </c>
+    </row>
+    <row r="78" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>282</v>
       </c>
@@ -6750,8 +7001,11 @@
       <c r="V78" s="7">
         <v>-130.01348899999999</v>
       </c>
-    </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W78" s="10">
+        <v>45126</v>
+      </c>
+    </row>
+    <row r="79" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>285</v>
       </c>
@@ -6818,8 +7072,11 @@
       <c r="V79" s="7">
         <v>-130.01348899999999</v>
       </c>
-    </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W79" s="10">
+        <v>45126</v>
+      </c>
+    </row>
+    <row r="80" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>287</v>
       </c>
@@ -6886,8 +7143,11 @@
       <c r="V80" s="7">
         <v>-130.01348899999999</v>
       </c>
-    </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W80" s="10">
+        <v>45126</v>
+      </c>
+    </row>
+    <row r="81" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>289</v>
       </c>
@@ -6954,8 +7214,11 @@
       <c r="V81" s="7">
         <v>-130.01348899999999</v>
       </c>
-    </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W81" s="10">
+        <v>45126</v>
+      </c>
+    </row>
+    <row r="82" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>291</v>
       </c>
@@ -7022,8 +7285,11 @@
       <c r="V82" s="7">
         <v>-130.01348899999999</v>
       </c>
-    </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W82" s="10">
+        <v>45126</v>
+      </c>
+    </row>
+    <row r="83" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>293</v>
       </c>
@@ -7090,8 +7356,11 @@
       <c r="V83" s="7">
         <v>-130.01348899999999</v>
       </c>
-    </row>
-    <row r="84" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W83" s="10">
+        <v>45126</v>
+      </c>
+    </row>
+    <row r="84" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>295</v>
       </c>
@@ -7158,8 +7427,11 @@
       <c r="V84" s="7">
         <v>-130.01348899999999</v>
       </c>
-    </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W84" s="10">
+        <v>45126</v>
+      </c>
+    </row>
+    <row r="85" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>297</v>
       </c>
@@ -7226,8 +7498,11 @@
       <c r="V85" s="7">
         <v>-130.01348899999999</v>
       </c>
-    </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W85" s="10">
+        <v>45126</v>
+      </c>
+    </row>
+    <row r="86" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>299</v>
       </c>
@@ -7294,8 +7569,11 @@
       <c r="V86" s="7">
         <v>-130.04949999999999</v>
       </c>
-    </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W86" s="10">
+        <v>45128</v>
+      </c>
+    </row>
+    <row r="87" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>301</v>
       </c>
@@ -7362,8 +7640,11 @@
       <c r="V87" s="7">
         <v>-130.04949999999999</v>
       </c>
-    </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W87" s="10">
+        <v>45128</v>
+      </c>
+    </row>
+    <row r="88" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>303</v>
       </c>
@@ -7430,8 +7711,11 @@
       <c r="V88" s="7">
         <v>-130.04949999999999</v>
       </c>
-    </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W88" s="10">
+        <v>45128</v>
+      </c>
+    </row>
+    <row r="89" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>306</v>
       </c>
@@ -7498,8 +7782,11 @@
       <c r="V89" s="6">
         <v>-129.97996670000001</v>
       </c>
-    </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W89" s="10">
+        <v>45129</v>
+      </c>
+    </row>
+    <row r="90" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>308</v>
       </c>
@@ -7566,8 +7853,11 @@
       <c r="V90" s="6">
         <v>-129.97996670000001</v>
       </c>
-    </row>
-    <row r="91" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W90" s="10">
+        <v>45129</v>
+      </c>
+    </row>
+    <row r="91" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>310</v>
       </c>
@@ -7634,8 +7924,14 @@
       <c r="V91" s="6">
         <v>-129.97996670000001</v>
       </c>
+      <c r="W91" s="10">
+        <v>45129</v>
+      </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:V91">
+    <sortCondition ref="B2:B91"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>